<commit_message>
Application du nouveau thèmes et corrections QA 3e36fff7efc9e5c3030998c5a2aa599e9315d4ba
</commit_message>
<xml_diff>
--- a/nmoreau/ig/CodeSystem-document-type-cs.xlsx
+++ b/nmoreau/ig/CodeSystem-document-type-cs.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.2.0</t>
+    <t>0.1.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-11-19T09:47:12+00:00</t>
+    <t>2026-01-14T12:51:21+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
#12 #18 Correction sur l'extension AMC afin d'être multi domaine + utilisation du FR Core 2.2.0 f6338579ae703322d3d922e651e1f0610f806fdf
</commit_message>
<xml_diff>
--- a/nmoreau/ig/CodeSystem-document-type-cs.xlsx
+++ b/nmoreau/ig/CodeSystem-document-type-cs.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.0</t>
+    <t>1.0.0-ballot</t>
   </si>
   <si>
     <t>Name</t>
@@ -48,7 +48,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>draft</t>
+    <t>active</t>
   </si>
   <si>
     <t>Experimental</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-24T09:27:09+00:00</t>
+    <t>2026-04-10T11:37:26+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>